<commit_message>
Leads: 2026-10-30 15:11 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://www.tenpennyhvactn.com/installation</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>leetenpenny@yahoo.com</t>
@@ -614,6 +613,62 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Plumbing &amp; Heating | Casper, WY | Davidson Mechanical</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>davidsonmechanical.net</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.davidsonmechanical.net/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>td@davidsonmechanical.net</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(307) 577-4000</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Casper WY</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>86</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>plumbing company Casper WY</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 15:13 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,6 @@
           <t>https://www.davidsonmechanical.net/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>td@davidsonmechanical.net</t>
@@ -669,6 +668,66 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Advosy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>advosy.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://advosy.com/roofing/henderson</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Services Areas</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>hello@advosy.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(480) 637-5224</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Henderson NV</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>88</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofer Henderson NV</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 17:08 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -733,6 +733,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MBR Construction Services</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>constructwithmbr.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.constructwithmbr.com/services/emergency-plumbing</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sapphire Dr</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>plumbing@mbrconstruction.net</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(435) 218-6186</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>emergency plumber St George UT</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:23 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -793,6 +793,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Culture Construction</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cultureccc.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://cultureccc.com/services/roofing/residential/services-in-waukegan-illinois</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Project Details</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@cultureccc.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(234) 285-8873</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Waukegan IL</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roof replacement Waukegan IL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:26 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -853,6 +853,62 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dierna Contracting, LLC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>metalroofrepairrochester.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>http://www.metalroofrepairrochester.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofrepairrochester.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>585-206-4848</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>84</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Rochester NY</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:27 UTC (cycle 185)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -874,7 +874,6 @@
           <t>http://www.metalroofrepairrochester.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>moreinfo@metalroofrepairrochester.com</t>
@@ -904,6 +903,66 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>McCall's Air Conditioning and Heating</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>mccallsac.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.mccallsac.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Why East</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>office@mccallsac.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>480-396-0041</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>heating and cooling company Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:29 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Premier Roofing &amp; Contracting - Highly-Rated &amp; Trusted Roofing Company</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>premierroofingandcontracting.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.premierroofingandcontracting.com/near-me/best-san-marcos-roofer-premier-roofing/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Serving Our</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@4premierroofs.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>210-867-6001</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:30 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1028,6 +1028,62 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Port St Lucie Plumbing Inc: Trusted plumbing services in Port St. Lucie</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>portstlucieplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.portstlucieplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>portstlucieplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(772) 468-6524</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>84</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>plumbing company Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:35 UTC (cycle 190)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1049,7 +1049,6 @@
           <t>https://www.portstlucieplumbinginc.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>portstlucieplumbing@gmail.com</t>
@@ -1079,6 +1078,126 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Top Notch Well Pumps &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>choosetopnotch.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.choosetopnotch.com/water-heater-repair-replacement</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Why Dayton</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>service@choosetopnotch.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>937-421-8200</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>water heater repair Dayton OH</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Water Heater Repair | Guardian Plumbing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>guardianplumbingoh.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://guardianplumbingoh.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>contact@guardianplumbingoh.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>937-818-1123</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>water heater repair Dayton OH</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:36 UTC (cycle 191)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Infinite Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>infroofing.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.infroofing.com/roofing-stockton/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Verifiable Reviews</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@infroofing.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(559) 550-6398</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof replacement Stockton CA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:38 UTC (cycle 192)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1263,6 +1263,122 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Licensed Plumbers in Lawrence, KS | Expert Plumbing Repairs</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>avidplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.avidplumbingllc.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>avidplumbingks@gmail.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>785-379-1710</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Lawrence KS</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>plumber Lawrence KS</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Plumbers of Greensboro</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>plumbersofgreensboro.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://plumbersofgreensboro.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>plumbersofgreensboronc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>877 708 6986</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Greensboro NC</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>emergency plumber Greensboro NC</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:39 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1284,7 +1284,6 @@
           <t>https://www.avidplumbingllc.com/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>avidplumbingks@gmail.com</t>
@@ -1374,6 +1373,66 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Calderon HVAC and Plumbing Inc</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>calderonhvac.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://calderonhvac.com/service-areas/hvac-contractor-high-point-nc/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Barrington Oaks</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>filiberto@calderoncorps.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>336-964-3611</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>HVAC contractor High Point NC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:41 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1438,6 +1438,126 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Quik Plumbing Sewer &amp; Drain</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>quikplumbers.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://quikplumbers.com/services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Quik Plumbing</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>quikplumbinginc@gmail.co</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>864-546-9959</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>sewer repair Greenville SC</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lafayette, LA | Roofing Company | Fontenot &amp; Sons Roofers Inc.</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>fontenotandsons.net</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.fontenotandsons.net/lafayette--la</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>At Fontenot</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>fontenot.r@att.net</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>318-240-9840</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>98</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roof repair company Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 19:42 UTC (cycle 195)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1558,6 +1558,62 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AC Installation Houston TX | New HVAC System Replacement</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>atlasacandheat.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://atlasacandheat.com/services/ac-installation</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@atlasacandheat.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(713) 478-5655</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>AC installation Houston TX</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:37 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1579,7 +1579,6 @@
           <t>https://atlasacandheat.com/services/ac-installation</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>info@atlasacandheat.com</t>
@@ -1609,6 +1608,62 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Lehi, UT Roofer | Roof Repair &amp; Replacement</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>dynamic-roof.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.dynamic-roof.com/service-areas/lehi-ut</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@dynamic-roof.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(801) 783-4260</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Lehi UT</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roofer Lehi UT</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:40 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1634,7 +1634,6 @@
           <t>https://www.dynamic-roof.com/service-areas/lehi-ut</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>info@dynamic-roof.com</t>
@@ -1664,6 +1663,66 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Trinity Climate Control</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>trinityclimate.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.trinityclimate.com/service-area/norman/heating-repair</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Trinity Other</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>anthony@trinityclimate.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>405-420-4895</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Norman OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>furnace repair Norman OK</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:45 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1728,6 +1728,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ginisi Plumbing</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ginisiplumbing.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.ginisiplumbing.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Jon Lapierre</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>joe@ginisiplumbing.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(508) 208-7348</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>drain cleaning service Worcester MA</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:46 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1788,6 +1788,62 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tuccinardi Plumbing &amp; Heating Inc. | Plumbers | Stamford, CT</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>tuccinardiplumbing.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.tuccinardiplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>mtucc@aol.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>203-325-8247</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>86</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>plumber Stamford CT</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:48 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1809,7 +1809,6 @@
           <t>https://www.tuccinardiplumbing.com/</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>mtucc@aol.com</t>
@@ -1839,6 +1838,122 @@
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Plumbing | Great Falls, MT | Central Plumbing, Heating, Excavation</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>centralph.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.centralph.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Mike Waldenberg</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>pat.bahnmiller@centralph.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>406-388-1000</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Great Falls MT</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>98</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>plumbing company Great Falls MT</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Augusta Evans Lincolnton Richmond County Georgia Roofing Contractor Repair Servi</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>roofingservicesofaugusta.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.roofingservicesofaugusta.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>roofingservicesaugusta@gmail.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>706-814-3207</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Augusta GA</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>78</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>roofing contractor Augusta GA</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:49 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1924,7 +1924,6 @@
           <t>https://www.roofingservicesofaugusta.com/</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>roofingservicesaugusta@gmail.com</t>
@@ -1954,6 +1953,126 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ohio's Leading Roofing Specialists | Absolute Roofing</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>absoluteroofing.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://absoluteroofing.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Letter From</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>info@absoluteroofing.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>216-898-1563</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Cleveland OH</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>96</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>roofer Cleveland OH</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Wollman Construction</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>wollmanconstruction.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://wollmanconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Wollman Construction</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>info@wollmanconstruction.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>605.261.5335</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>94</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>roofing contractor Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:51 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2078,6 +2078,66 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>KanMo Roofing</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>kanmoroofing.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.kanmoroofing.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>General Cont</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>justin@kanmoroofing.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>913-608-8099</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Kansas City MO</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>98</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roofer Kansas City MO</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-30 20:52 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-30.xlsx
+++ b/output/leads_2026-10-30.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2138,6 +2138,66 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>New England Ductless</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>newenglandductless.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://newenglandductless.com/plumbing-services/water-heater/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Greater Boston</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@neductless.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(617) 915-2803</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>water heater repair Boston MA</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>